<commit_message>
using 2025-11-03 revised spreadsheet from Charli Morgan that has field coordinates entered and I renamed wq field names so they could be read into R
</commit_message>
<xml_diff>
--- a/survey_wqdata/SR_Data.xlsx
+++ b/survey_wqdata/SR_Data.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArcGIS\Documents\nokuse_seven_runs_survey\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArcGIS\Documents\nokuse_seven_runs_survey_old\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5BD0269-F7D7-43C3-BF28-E15EB0BD0860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1FDADF7-C335-49B9-9A98-6424F1134054}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="17400" yWindow="885" windowWidth="20115" windowHeight="19680" xr2:uid="{BC263282-6D8F-47C7-8BF3-A88688F790FA}"/>
+    <workbookView xWindow="480" yWindow="1695" windowWidth="19275" windowHeight="19680" xr2:uid="{BC263282-6D8F-47C7-8BF3-A88688F790FA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AA$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AC$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="68">
   <si>
     <t>Site</t>
   </si>
@@ -269,6 +269,12 @@
   </si>
   <si>
     <t>Dip net x10: crayfish, Gambusia, dragonfly larvae</t>
+  </si>
+  <si>
+    <t>Field Latitude</t>
+  </si>
+  <si>
+    <t>Field Longitude</t>
   </si>
 </sst>
 </file>
@@ -325,11 +331,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -664,22 +671,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22E256C1-2401-41CC-88F3-2A60CDB12830}">
-  <dimension ref="A1:AB21"/>
+  <dimension ref="A1:AD21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14.7109375" customWidth="1"/>
     <col min="3" max="3" width="9.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.140625" customWidth="1"/>
-    <col min="6" max="6" width="11.85546875" customWidth="1"/>
-    <col min="9" max="9" width="10.28515625" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
-    <col min="12" max="12" width="11.140625" customWidth="1"/>
-    <col min="13" max="13" width="13.7109375" customWidth="1"/>
-    <col min="14" max="14" width="12.28515625" customWidth="1"/>
-    <col min="15" max="16" width="10.7109375" customWidth="1"/>
+    <col min="6" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="10.28515625" customWidth="1"/>
+    <col min="13" max="13" width="14" customWidth="1"/>
+    <col min="14" max="14" width="11.140625" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" customWidth="1"/>
+    <col min="16" max="16" width="12.28515625" customWidth="1"/>
+    <col min="17" max="18" width="10.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:30" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -699,73 +706,79 @@
         <v>25</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="W1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -784,74 +797,74 @@
       <c r="F2">
         <v>-86.038640000000001</v>
       </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>51</v>
       </c>
-      <c r="H2">
+      <c r="J2">
         <v>0.25</v>
       </c>
-      <c r="I2">
+      <c r="K2">
         <v>22.7</v>
       </c>
-      <c r="J2">
+      <c r="L2">
         <v>5.08</v>
       </c>
-      <c r="K2">
+      <c r="M2">
         <v>7.71</v>
       </c>
-      <c r="L2">
+      <c r="N2">
         <v>89.5</v>
       </c>
-      <c r="M2">
+      <c r="O2">
         <v>17.600000000000001</v>
       </c>
-      <c r="N2">
+      <c r="P2">
         <v>0.01</v>
       </c>
-      <c r="O2">
+      <c r="Q2">
         <v>1.63</v>
       </c>
-      <c r="P2" t="s">
+      <c r="R2" t="s">
         <v>52</v>
       </c>
-      <c r="Q2">
+      <c r="S2">
         <v>1.37</v>
       </c>
-      <c r="R2">
+      <c r="T2">
         <v>1.63</v>
       </c>
-      <c r="S2">
+      <c r="U2">
         <v>0.34</v>
       </c>
-      <c r="T2">
+      <c r="V2">
         <v>99.48</v>
       </c>
-      <c r="U2" t="s">
-        <v>47</v>
-      </c>
-      <c r="V2" t="s">
-        <v>47</v>
-      </c>
       <c r="W2" t="s">
+        <v>47</v>
+      </c>
+      <c r="X2" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y2" t="s">
         <v>49</v>
       </c>
-      <c r="X2" t="s">
+      <c r="Z2" t="s">
         <v>48</v>
       </c>
-      <c r="Y2" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>47</v>
-      </c>
       <c r="AA2" t="s">
         <v>47</v>
       </c>
       <c r="AB2" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>47</v>
+      </c>
+      <c r="AD2" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -870,71 +883,71 @@
       <c r="F3">
         <v>-86.028282000000004</v>
       </c>
-      <c r="G3" t="s">
+      <c r="I3" t="s">
         <v>51</v>
       </c>
-      <c r="H3">
+      <c r="J3">
         <v>0.38</v>
       </c>
-      <c r="I3">
+      <c r="K3">
         <v>25.6</v>
       </c>
-      <c r="J3">
+      <c r="L3">
         <v>5.39</v>
       </c>
-      <c r="K3">
+      <c r="M3">
         <v>7.93</v>
       </c>
-      <c r="L3">
+      <c r="N3">
         <v>97.1</v>
       </c>
-      <c r="M3">
+      <c r="O3">
         <v>18.100000000000001</v>
       </c>
-      <c r="N3">
+      <c r="P3">
         <v>0.01</v>
       </c>
-      <c r="O3">
+      <c r="Q3">
         <v>2.56</v>
       </c>
-      <c r="P3" t="s">
+      <c r="R3" t="s">
         <v>52</v>
       </c>
-      <c r="Q3">
+      <c r="S3">
         <v>2.69</v>
       </c>
-      <c r="R3">
+      <c r="T3">
         <v>2.9</v>
       </c>
-      <c r="S3">
+      <c r="U3">
         <v>0.13</v>
       </c>
-      <c r="T3">
+      <c r="V3">
         <v>95.84</v>
       </c>
-      <c r="U3" t="s">
-        <v>47</v>
-      </c>
-      <c r="V3" t="s">
-        <v>47</v>
-      </c>
       <c r="W3" t="s">
+        <v>47</v>
+      </c>
+      <c r="X3" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y3" t="s">
         <v>49</v>
       </c>
-      <c r="X3" t="s">
+      <c r="Z3" t="s">
         <v>48</v>
       </c>
-      <c r="Y3" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>47</v>
-      </c>
       <c r="AA3" t="s">
         <v>47</v>
       </c>
+      <c r="AB3" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -953,74 +966,74 @@
       <c r="F4">
         <v>-86.016197000000005</v>
       </c>
-      <c r="G4" t="s">
+      <c r="I4" t="s">
         <v>51</v>
       </c>
-      <c r="H4">
+      <c r="J4">
         <v>0.4</v>
       </c>
-      <c r="I4">
+      <c r="K4">
         <v>22.5</v>
       </c>
-      <c r="J4">
+      <c r="L4">
         <v>5.01</v>
       </c>
-      <c r="K4">
+      <c r="M4">
         <v>8.0299999999999994</v>
       </c>
-      <c r="L4">
+      <c r="N4">
         <v>92.7</v>
       </c>
-      <c r="M4">
+      <c r="O4">
         <v>19.100000000000001</v>
       </c>
-      <c r="N4">
+      <c r="P4">
         <v>0.01</v>
       </c>
-      <c r="O4">
+      <c r="Q4">
         <v>2.14</v>
       </c>
-      <c r="P4" t="s">
+      <c r="R4" t="s">
         <v>52</v>
       </c>
-      <c r="Q4">
+      <c r="S4">
         <v>4.83</v>
       </c>
-      <c r="R4">
+      <c r="T4">
         <v>6.04</v>
       </c>
-      <c r="S4">
+      <c r="U4">
         <v>0.27</v>
       </c>
-      <c r="T4">
+      <c r="V4">
         <v>99.48</v>
       </c>
-      <c r="U4" t="s">
-        <v>47</v>
-      </c>
-      <c r="V4" t="s">
-        <v>47</v>
-      </c>
       <c r="W4" t="s">
+        <v>47</v>
+      </c>
+      <c r="X4" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y4" t="s">
         <v>49</v>
       </c>
-      <c r="X4" t="s">
+      <c r="Z4" t="s">
         <v>48</v>
       </c>
-      <c r="Y4" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z4" t="s">
-        <v>47</v>
-      </c>
       <c r="AA4" t="s">
         <v>47</v>
       </c>
       <c r="AB4" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>47</v>
+      </c>
+      <c r="AD4" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1039,71 +1052,71 @@
       <c r="F5">
         <v>-85.978043</v>
       </c>
-      <c r="G5" t="s">
+      <c r="I5" t="s">
         <v>51</v>
       </c>
-      <c r="H5">
+      <c r="J5">
         <v>0.32</v>
       </c>
-      <c r="I5">
+      <c r="K5">
         <v>20.6</v>
       </c>
-      <c r="J5">
+      <c r="L5">
         <v>5.64</v>
       </c>
-      <c r="K5">
+      <c r="M5">
         <v>8.4700000000000006</v>
       </c>
-      <c r="L5">
+      <c r="N5">
         <v>94.4</v>
       </c>
-      <c r="M5">
+      <c r="O5">
         <v>19.100000000000001</v>
       </c>
-      <c r="N5">
+      <c r="P5">
         <v>0.01</v>
       </c>
-      <c r="O5">
+      <c r="Q5">
         <v>2.5099999999999998</v>
       </c>
-      <c r="P5" t="s">
+      <c r="R5" t="s">
         <v>52</v>
       </c>
-      <c r="Q5">
+      <c r="S5">
         <v>6.45</v>
       </c>
-      <c r="R5">
+      <c r="T5">
         <v>7.06</v>
       </c>
-      <c r="S5">
+      <c r="U5">
         <v>0.37</v>
       </c>
-      <c r="T5">
+      <c r="V5">
         <v>84.92</v>
       </c>
-      <c r="U5" t="s">
-        <v>47</v>
-      </c>
-      <c r="V5" t="s">
-        <v>47</v>
-      </c>
       <c r="W5" t="s">
+        <v>47</v>
+      </c>
+      <c r="X5" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y5" t="s">
         <v>49</v>
       </c>
-      <c r="X5" t="s">
+      <c r="Z5" t="s">
         <v>48</v>
       </c>
-      <c r="Y5" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z5" t="s">
-        <v>47</v>
-      </c>
       <c r="AA5" t="s">
         <v>47</v>
       </c>
+      <c r="AB5" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1122,71 +1135,77 @@
       <c r="F6">
         <v>-85.963539999999995</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6">
+        <v>30.556778000000001</v>
+      </c>
+      <c r="H6">
+        <v>-85.963860999999994</v>
+      </c>
+      <c r="I6" t="s">
         <v>51</v>
       </c>
-      <c r="H6">
+      <c r="J6">
         <v>0.32</v>
       </c>
-      <c r="I6">
+      <c r="K6">
         <v>21.8</v>
       </c>
-      <c r="J6">
+      <c r="L6">
         <v>5.55</v>
       </c>
-      <c r="K6">
+      <c r="M6">
         <v>8.33</v>
       </c>
-      <c r="L6">
+      <c r="N6">
         <v>94.9</v>
       </c>
-      <c r="M6">
+      <c r="O6">
         <v>19.100000000000001</v>
       </c>
-      <c r="N6">
+      <c r="P6">
         <v>0.01</v>
       </c>
-      <c r="O6">
+      <c r="Q6">
         <v>3.71</v>
       </c>
-      <c r="P6" t="s">
+      <c r="R6" t="s">
         <v>52</v>
       </c>
-      <c r="Q6">
+      <c r="S6">
         <v>5.13</v>
       </c>
-      <c r="R6">
+      <c r="T6">
         <v>6.37</v>
       </c>
-      <c r="S6">
+      <c r="U6">
         <v>0.41</v>
       </c>
-      <c r="T6">
+      <c r="V6">
         <v>96.1</v>
       </c>
-      <c r="U6" t="s">
-        <v>47</v>
-      </c>
-      <c r="V6" t="s">
-        <v>47</v>
-      </c>
       <c r="W6" t="s">
+        <v>47</v>
+      </c>
+      <c r="X6" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y6" t="s">
         <v>49</v>
       </c>
-      <c r="X6" t="s">
+      <c r="Z6" t="s">
         <v>48</v>
       </c>
-      <c r="Y6" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z6" t="s">
-        <v>47</v>
-      </c>
       <c r="AA6" t="s">
         <v>47</v>
       </c>
+      <c r="AB6" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -1205,71 +1224,71 @@
       <c r="F7">
         <v>-85.962569000000002</v>
       </c>
-      <c r="G7" t="s">
+      <c r="I7" t="s">
         <v>51</v>
       </c>
-      <c r="H7">
+      <c r="J7">
         <v>0.43</v>
       </c>
-      <c r="I7">
+      <c r="K7">
         <v>21.6</v>
       </c>
-      <c r="J7">
+      <c r="L7">
         <v>5.6</v>
       </c>
-      <c r="K7">
+      <c r="M7">
         <v>8.3000000000000007</v>
       </c>
-      <c r="L7">
+      <c r="N7">
         <v>94.2</v>
       </c>
-      <c r="M7">
+      <c r="O7">
         <v>19.100000000000001</v>
       </c>
-      <c r="N7">
+      <c r="P7">
         <v>0.01</v>
       </c>
-      <c r="O7">
+      <c r="Q7">
         <v>2.33</v>
       </c>
-      <c r="P7" t="s">
+      <c r="R7" t="s">
         <v>52</v>
       </c>
-      <c r="Q7">
+      <c r="S7">
         <v>4.83</v>
       </c>
-      <c r="R7">
+      <c r="T7">
         <v>6.81</v>
       </c>
-      <c r="S7">
+      <c r="U7">
         <v>0.71</v>
       </c>
-      <c r="T7">
+      <c r="V7">
         <v>92.72</v>
       </c>
-      <c r="U7" t="s">
-        <v>47</v>
-      </c>
-      <c r="V7" t="s">
-        <v>47</v>
-      </c>
       <c r="W7" t="s">
+        <v>47</v>
+      </c>
+      <c r="X7" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y7" t="s">
         <v>49</v>
       </c>
-      <c r="X7" t="s">
+      <c r="Z7" t="s">
         <v>48</v>
       </c>
-      <c r="Y7" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z7" t="s">
-        <v>47</v>
-      </c>
       <c r="AA7" t="s">
         <v>47</v>
       </c>
+      <c r="AB7" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC7" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -1282,77 +1301,83 @@
       <c r="D8" s="3">
         <v>0.37986111111111109</v>
       </c>
-      <c r="E8">
+      <c r="E8" s="4">
         <v>30.581834000000001</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="4">
         <v>-85.979294999999993</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="4">
+        <v>30.581028</v>
+      </c>
+      <c r="H8" s="4">
+        <v>-85.979388999999998</v>
+      </c>
+      <c r="I8" t="s">
         <v>51</v>
       </c>
-      <c r="H8">
+      <c r="J8">
         <v>0.32</v>
       </c>
-      <c r="I8">
+      <c r="K8">
         <v>21.9</v>
       </c>
-      <c r="J8">
+      <c r="L8">
         <v>6.32</v>
       </c>
-      <c r="K8">
+      <c r="M8">
         <v>7.68</v>
       </c>
-      <c r="L8">
+      <c r="N8">
         <v>87.7</v>
       </c>
-      <c r="M8">
+      <c r="O8">
         <v>39.200000000000003</v>
       </c>
-      <c r="N8">
+      <c r="P8">
         <v>0.02</v>
       </c>
-      <c r="O8">
+      <c r="Q8">
         <v>1.44</v>
       </c>
-      <c r="P8" t="s">
+      <c r="R8" t="s">
         <v>52</v>
       </c>
-      <c r="Q8">
+      <c r="S8">
         <v>1.65</v>
       </c>
-      <c r="R8">
+      <c r="T8">
         <v>2.36</v>
       </c>
-      <c r="S8">
+      <c r="U8">
         <v>0.06</v>
       </c>
-      <c r="T8">
+      <c r="V8">
         <v>97.92</v>
       </c>
-      <c r="U8" t="s">
-        <v>47</v>
-      </c>
-      <c r="V8" t="s">
-        <v>47</v>
-      </c>
       <c r="W8" t="s">
+        <v>47</v>
+      </c>
+      <c r="X8" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y8" t="s">
         <v>49</v>
       </c>
-      <c r="X8" t="s">
+      <c r="Z8" t="s">
         <v>48</v>
       </c>
-      <c r="Y8" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z8" t="s">
-        <v>47</v>
-      </c>
       <c r="AA8" t="s">
         <v>47</v>
       </c>
+      <c r="AB8" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC8" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -1365,77 +1390,83 @@
       <c r="D9" s="3">
         <v>0.39791666666666664</v>
       </c>
-      <c r="E9">
+      <c r="E9" s="4">
         <v>30.579967</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="4">
         <v>-85.980097000000001</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="4">
+        <v>30.579861000000001</v>
+      </c>
+      <c r="H9" s="4">
+        <v>-85.979889</v>
+      </c>
+      <c r="I9" t="s">
         <v>51</v>
       </c>
-      <c r="H9">
+      <c r="J9">
         <v>0.25</v>
       </c>
-      <c r="I9">
+      <c r="K9">
         <v>21.9</v>
       </c>
-      <c r="J9">
+      <c r="L9">
         <v>6.39</v>
       </c>
-      <c r="K9">
+      <c r="M9">
         <v>7.94</v>
       </c>
-      <c r="L9">
+      <c r="N9">
         <v>90.7</v>
       </c>
-      <c r="M9">
+      <c r="O9">
         <v>38.4</v>
       </c>
-      <c r="N9">
+      <c r="P9">
         <v>0.02</v>
       </c>
-      <c r="O9">
+      <c r="Q9">
         <v>1.74</v>
       </c>
-      <c r="P9" t="s">
+      <c r="R9" t="s">
         <v>52</v>
       </c>
-      <c r="Q9">
+      <c r="S9">
         <v>1.0900000000000001</v>
       </c>
-      <c r="R9">
+      <c r="T9">
         <v>1.83</v>
       </c>
-      <c r="S9">
+      <c r="U9">
         <v>0.08</v>
       </c>
-      <c r="T9">
+      <c r="V9">
         <v>100</v>
       </c>
-      <c r="U9" t="s">
-        <v>47</v>
-      </c>
-      <c r="V9" t="s">
-        <v>47</v>
-      </c>
       <c r="W9" t="s">
+        <v>47</v>
+      </c>
+      <c r="X9" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y9" t="s">
         <v>49</v>
       </c>
-      <c r="X9" t="s">
+      <c r="Z9" t="s">
         <v>48</v>
       </c>
-      <c r="Y9" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z9" t="s">
-        <v>47</v>
-      </c>
       <c r="AA9" t="s">
         <v>47</v>
       </c>
+      <c r="AB9" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC9" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -1448,80 +1479,86 @@
       <c r="D10" s="3">
         <v>0.52152777777777781</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="4">
         <v>30.569496000000001</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="4">
         <v>-85.979523</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="4">
+        <v>30.569500000000001</v>
+      </c>
+      <c r="H10" s="4">
+        <v>-85.979528000000002</v>
+      </c>
+      <c r="I10" t="s">
         <v>51</v>
       </c>
-      <c r="H10">
+      <c r="J10">
         <v>0.25</v>
       </c>
-      <c r="I10">
+      <c r="K10">
         <v>22.6</v>
       </c>
-      <c r="J10">
+      <c r="L10">
         <v>6.37</v>
       </c>
-      <c r="K10">
+      <c r="M10">
         <v>7.69</v>
       </c>
-      <c r="L10">
+      <c r="N10">
         <v>89.1</v>
       </c>
-      <c r="M10">
+      <c r="O10">
         <v>22.2</v>
       </c>
-      <c r="N10">
+      <c r="P10">
         <v>0.01</v>
       </c>
-      <c r="O10">
+      <c r="Q10">
         <v>2.2999999999999998</v>
       </c>
-      <c r="P10" t="s">
+      <c r="R10" t="s">
         <v>52</v>
       </c>
-      <c r="Q10">
+      <c r="S10">
         <v>2.82</v>
       </c>
-      <c r="R10">
+      <c r="T10">
         <v>3.56</v>
       </c>
-      <c r="S10">
+      <c r="U10">
         <v>0.22</v>
       </c>
-      <c r="T10">
+      <c r="V10">
         <v>98.18</v>
       </c>
-      <c r="U10" t="s">
-        <v>47</v>
-      </c>
-      <c r="V10" t="s">
-        <v>47</v>
-      </c>
       <c r="W10" t="s">
+        <v>47</v>
+      </c>
+      <c r="X10" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y10" t="s">
         <v>49</v>
       </c>
-      <c r="X10" t="s">
+      <c r="Z10" t="s">
         <v>48</v>
       </c>
-      <c r="Y10" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z10" t="s">
+      <c r="AA10" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB10" t="s">
         <v>61</v>
       </c>
-      <c r="AA10" t="s">
-        <v>47</v>
-      </c>
-      <c r="AB10" t="s">
+      <c r="AC10" t="s">
+        <v>47</v>
+      </c>
+      <c r="AD10" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -1534,81 +1571,87 @@
       <c r="D11" t="s">
         <v>60</v>
       </c>
-      <c r="E11">
+      <c r="E11" s="4">
         <v>30.567005999999999</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="4">
         <f>F29-85.979297</f>
         <v>-85.979297000000003</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="4">
+        <v>30.566330000000001</v>
+      </c>
+      <c r="H11" s="4">
+        <v>-85.97851</v>
+      </c>
+      <c r="I11" t="s">
         <v>51</v>
       </c>
-      <c r="H11">
+      <c r="J11">
         <v>0.34</v>
       </c>
-      <c r="I11">
+      <c r="K11">
         <v>23</v>
       </c>
-      <c r="J11">
+      <c r="L11">
         <v>5.86</v>
       </c>
-      <c r="K11">
+      <c r="M11">
         <v>7.65</v>
       </c>
-      <c r="L11">
+      <c r="N11">
         <v>89.1</v>
       </c>
-      <c r="M11">
+      <c r="O11">
         <v>22.1</v>
       </c>
-      <c r="N11">
+      <c r="P11">
         <v>0.01</v>
       </c>
-      <c r="O11">
+      <c r="Q11">
         <v>3.08</v>
       </c>
-      <c r="P11" t="s">
+      <c r="R11" t="s">
         <v>52</v>
       </c>
-      <c r="Q11">
+      <c r="S11">
         <v>2.11</v>
       </c>
-      <c r="R11">
+      <c r="T11">
         <v>3.25</v>
       </c>
-      <c r="S11">
+      <c r="U11">
         <v>0.13</v>
       </c>
-      <c r="T11">
+      <c r="V11">
         <v>98.44</v>
       </c>
-      <c r="U11" t="s">
-        <v>47</v>
-      </c>
-      <c r="V11" t="s">
-        <v>47</v>
-      </c>
       <c r="W11" t="s">
+        <v>47</v>
+      </c>
+      <c r="X11" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y11" t="s">
         <v>49</v>
       </c>
-      <c r="X11" t="s">
+      <c r="Z11" t="s">
         <v>48</v>
       </c>
-      <c r="Y11" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z11" t="s">
+      <c r="AA11" t="s">
+        <v>47</v>
+      </c>
+      <c r="AB11" t="s">
         <v>61</v>
       </c>
-      <c r="AA11" t="s">
-        <v>47</v>
-      </c>
-      <c r="AB11" t="s">
+      <c r="AC11" t="s">
+        <v>47</v>
+      </c>
+      <c r="AD11" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -1621,77 +1664,83 @@
       <c r="D12" s="3">
         <v>0.43472222222222223</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="4">
         <v>30.580921</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="4">
         <v>-85.964935999999994</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="4">
+        <v>30.580943999999999</v>
+      </c>
+      <c r="H12" s="4">
+        <v>-85.965056000000004</v>
+      </c>
+      <c r="I12" t="s">
         <v>51</v>
       </c>
-      <c r="H12">
+      <c r="J12">
         <v>0.23</v>
       </c>
-      <c r="I12">
+      <c r="K12">
         <v>22</v>
       </c>
-      <c r="J12">
+      <c r="L12">
         <v>4.82</v>
       </c>
-      <c r="K12">
+      <c r="M12">
         <v>7.02</v>
       </c>
-      <c r="L12">
+      <c r="N12">
         <v>80.400000000000006</v>
       </c>
-      <c r="M12">
+      <c r="O12">
         <v>22.6</v>
       </c>
-      <c r="N12">
+      <c r="P12">
         <v>0.01</v>
       </c>
-      <c r="O12">
+      <c r="Q12">
         <v>2</v>
       </c>
-      <c r="P12" t="s">
+      <c r="R12" t="s">
         <v>52</v>
       </c>
-      <c r="Q12">
+      <c r="S12">
         <v>1.4</v>
       </c>
-      <c r="R12">
+      <c r="T12">
         <v>2</v>
       </c>
-      <c r="S12">
+      <c r="U12">
         <v>0.13</v>
       </c>
-      <c r="T12">
+      <c r="V12">
         <v>99.22</v>
       </c>
-      <c r="U12" t="s">
-        <v>47</v>
-      </c>
-      <c r="V12" t="s">
-        <v>47</v>
-      </c>
       <c r="W12" t="s">
+        <v>47</v>
+      </c>
+      <c r="X12" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y12" t="s">
         <v>49</v>
       </c>
-      <c r="X12" t="s">
+      <c r="Z12" t="s">
         <v>48</v>
       </c>
-      <c r="Y12" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z12" t="s">
-        <v>47</v>
-      </c>
       <c r="AA12" t="s">
         <v>47</v>
       </c>
+      <c r="AB12" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC12" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -1704,77 +1753,83 @@
       <c r="D13" s="3">
         <v>0.4777777777777778</v>
       </c>
-      <c r="E13">
+      <c r="E13" s="4">
         <v>30.570474999999998</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="4">
         <v>-85.966836999999998</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" s="4">
+        <v>30.570471999999999</v>
+      </c>
+      <c r="H13" s="4">
+        <v>-85.966333000000006</v>
+      </c>
+      <c r="I13" t="s">
         <v>51</v>
       </c>
-      <c r="H13">
+      <c r="J13">
         <v>0.31</v>
       </c>
-      <c r="I13">
+      <c r="K13">
         <v>22.6</v>
       </c>
-      <c r="J13">
+      <c r="L13">
         <v>5.0199999999999996</v>
       </c>
-      <c r="K13">
+      <c r="M13">
         <v>7.17</v>
       </c>
-      <c r="L13">
+      <c r="N13">
         <v>83</v>
       </c>
-      <c r="M13">
+      <c r="O13">
         <v>20.2</v>
       </c>
-      <c r="N13">
+      <c r="P13">
         <v>0.01</v>
       </c>
-      <c r="O13">
+      <c r="Q13">
         <v>2.48</v>
       </c>
-      <c r="P13" t="s">
+      <c r="R13" t="s">
         <v>52</v>
       </c>
-      <c r="Q13">
+      <c r="S13">
         <v>2.74</v>
       </c>
-      <c r="R13">
+      <c r="T13">
         <v>2.85</v>
       </c>
-      <c r="S13">
+      <c r="U13">
         <v>0.2</v>
       </c>
-      <c r="T13">
+      <c r="V13">
         <v>99.48</v>
       </c>
-      <c r="U13" t="s">
-        <v>47</v>
-      </c>
-      <c r="V13" t="s">
-        <v>47</v>
-      </c>
       <c r="W13" t="s">
+        <v>47</v>
+      </c>
+      <c r="X13" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y13" t="s">
         <v>49</v>
       </c>
-      <c r="X13" t="s">
+      <c r="Z13" t="s">
         <v>48</v>
       </c>
-      <c r="Y13" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z13" t="s">
-        <v>47</v>
-      </c>
       <c r="AA13" t="s">
         <v>47</v>
       </c>
+      <c r="AB13" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC13" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -1787,77 +1842,83 @@
       <c r="D14" s="3">
         <v>0.38055555555555554</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="4">
         <v>30.563506</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="4">
         <v>-85.966802999999999</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14" s="4">
+        <v>30.56325</v>
+      </c>
+      <c r="H14" s="4">
+        <v>-85.966443999999996</v>
+      </c>
+      <c r="I14" t="s">
         <v>51</v>
       </c>
-      <c r="H14">
+      <c r="J14">
         <v>0.3</v>
       </c>
-      <c r="I14">
+      <c r="K14">
         <v>20.8</v>
       </c>
-      <c r="J14">
+      <c r="L14">
         <v>5.0999999999999996</v>
       </c>
-      <c r="K14">
+      <c r="M14">
         <v>7.78</v>
       </c>
-      <c r="L14">
+      <c r="N14">
         <v>87.1</v>
       </c>
-      <c r="M14">
+      <c r="O14">
         <v>19.899999999999999</v>
       </c>
-      <c r="N14">
+      <c r="P14">
         <v>0.01</v>
       </c>
-      <c r="O14">
+      <c r="Q14">
         <v>1.85</v>
       </c>
-      <c r="P14" t="s">
+      <c r="R14" t="s">
         <v>52</v>
       </c>
-      <c r="Q14">
+      <c r="S14">
         <v>2.62</v>
       </c>
-      <c r="R14">
+      <c r="T14">
         <v>3</v>
       </c>
-      <c r="S14">
+      <c r="U14">
         <v>0.38</v>
       </c>
-      <c r="T14">
+      <c r="V14">
         <v>97.66</v>
       </c>
-      <c r="U14" t="s">
-        <v>47</v>
-      </c>
-      <c r="V14" t="s">
-        <v>47</v>
-      </c>
       <c r="W14" t="s">
+        <v>47</v>
+      </c>
+      <c r="X14" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y14" t="s">
         <v>49</v>
       </c>
-      <c r="X14" t="s">
+      <c r="Z14" t="s">
         <v>48</v>
       </c>
-      <c r="Y14" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z14" t="s">
-        <v>47</v>
-      </c>
       <c r="AA14" t="s">
         <v>47</v>
       </c>
+      <c r="AB14" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC14" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -1874,15 +1935,9 @@
       <c r="F15">
         <v>-85.984607999999994</v>
       </c>
-      <c r="G15" t="s">
+      <c r="I15" t="s">
         <v>51</v>
       </c>
-      <c r="H15" t="s">
-        <v>54</v>
-      </c>
-      <c r="I15" t="s">
-        <v>54</v>
-      </c>
       <c r="J15" t="s">
         <v>54</v>
       </c>
@@ -1938,10 +1993,16 @@
         <v>54</v>
       </c>
       <c r="AB15" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC15" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD15" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -1960,71 +2021,71 @@
       <c r="F16">
         <v>-85.981594000000001</v>
       </c>
-      <c r="G16" t="s">
+      <c r="I16" t="s">
         <v>51</v>
       </c>
-      <c r="H16">
+      <c r="J16">
         <v>0.22</v>
       </c>
-      <c r="I16">
+      <c r="K16">
         <v>20.7</v>
       </c>
-      <c r="J16">
+      <c r="L16">
         <v>5.94</v>
       </c>
-      <c r="K16">
+      <c r="M16">
         <v>8.58</v>
       </c>
-      <c r="L16">
+      <c r="N16">
         <v>95.6</v>
       </c>
-      <c r="M16">
+      <c r="O16">
         <v>21.9</v>
       </c>
-      <c r="N16">
+      <c r="P16">
         <v>0.01</v>
       </c>
-      <c r="O16">
+      <c r="Q16">
         <v>3.51</v>
       </c>
-      <c r="P16" t="s">
+      <c r="R16" t="s">
         <v>52</v>
       </c>
-      <c r="Q16">
+      <c r="S16">
         <v>2.72</v>
       </c>
-      <c r="R16">
+      <c r="T16">
         <v>2.97</v>
       </c>
-      <c r="S16">
+      <c r="U16">
         <v>0.41</v>
       </c>
-      <c r="T16">
+      <c r="V16">
         <v>98.18</v>
       </c>
-      <c r="U16" t="s">
-        <v>47</v>
-      </c>
-      <c r="V16" t="s">
-        <v>47</v>
-      </c>
       <c r="W16" t="s">
+        <v>47</v>
+      </c>
+      <c r="X16" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y16" t="s">
         <v>49</v>
       </c>
-      <c r="X16" t="s">
+      <c r="Z16" t="s">
         <v>48</v>
       </c>
-      <c r="Y16" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z16" t="s">
-        <v>47</v>
-      </c>
       <c r="AA16" t="s">
         <v>47</v>
       </c>
+      <c r="AB16" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC16" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="17" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -2043,15 +2104,9 @@
       <c r="F17">
         <v>-85.919370000000001</v>
       </c>
-      <c r="G17" t="s">
+      <c r="I17" t="s">
         <v>51</v>
       </c>
-      <c r="H17" t="s">
-        <v>54</v>
-      </c>
-      <c r="I17" t="s">
-        <v>54</v>
-      </c>
       <c r="J17" t="s">
         <v>54</v>
       </c>
@@ -2107,10 +2162,16 @@
         <v>54</v>
       </c>
       <c r="AB17" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC17" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD17" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -2129,74 +2190,74 @@
       <c r="F18">
         <v>-85.999088</v>
       </c>
-      <c r="G18" t="s">
+      <c r="I18" t="s">
         <v>51</v>
       </c>
-      <c r="H18">
+      <c r="J18">
         <v>0.36</v>
       </c>
-      <c r="I18">
+      <c r="K18">
         <v>22.3</v>
       </c>
-      <c r="J18">
+      <c r="L18">
         <v>4.8600000000000003</v>
       </c>
-      <c r="K18">
+      <c r="M18">
         <v>7.63</v>
       </c>
-      <c r="L18">
+      <c r="N18">
         <v>88</v>
       </c>
-      <c r="M18">
+      <c r="O18">
         <v>21.6</v>
       </c>
-      <c r="N18">
+      <c r="P18">
         <v>0.01</v>
       </c>
-      <c r="O18">
+      <c r="Q18">
         <v>2.82</v>
       </c>
-      <c r="P18" t="s">
+      <c r="R18" t="s">
         <v>52</v>
       </c>
-      <c r="Q18">
+      <c r="S18">
         <v>2.62</v>
       </c>
-      <c r="R18">
+      <c r="T18">
         <v>3.91</v>
       </c>
-      <c r="S18">
+      <c r="U18">
         <v>0.09</v>
       </c>
-      <c r="T18">
+      <c r="V18">
         <v>99.74</v>
       </c>
-      <c r="U18" t="s">
-        <v>47</v>
-      </c>
-      <c r="V18" t="s">
-        <v>47</v>
-      </c>
       <c r="W18" t="s">
+        <v>47</v>
+      </c>
+      <c r="X18" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y18" t="s">
         <v>49</v>
       </c>
-      <c r="X18" t="s">
+      <c r="Z18" t="s">
         <v>48</v>
       </c>
-      <c r="Y18" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z18" t="s">
-        <v>47</v>
-      </c>
       <c r="AA18" t="s">
         <v>47</v>
       </c>
       <c r="AB18" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC18" t="s">
+        <v>47</v>
+      </c>
+      <c r="AD18" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -2215,71 +2276,71 @@
       <c r="F19">
         <v>-85.935445999999999</v>
       </c>
-      <c r="G19" t="s">
+      <c r="I19" t="s">
         <v>51</v>
       </c>
-      <c r="H19">
+      <c r="J19">
         <v>0.3</v>
       </c>
-      <c r="I19">
+      <c r="K19">
         <v>21.8</v>
       </c>
-      <c r="J19">
+      <c r="L19">
         <v>5.38</v>
       </c>
-      <c r="K19">
+      <c r="M19">
         <v>7.72</v>
       </c>
-      <c r="L19">
+      <c r="N19">
         <v>88</v>
       </c>
-      <c r="M19">
+      <c r="O19">
         <v>21.3</v>
       </c>
-      <c r="N19">
+      <c r="P19">
         <v>0.01</v>
       </c>
-      <c r="O19">
+      <c r="Q19">
         <v>3.1</v>
       </c>
-      <c r="P19" t="s">
+      <c r="R19" t="s">
         <v>52</v>
       </c>
-      <c r="Q19">
+      <c r="S19">
         <v>2.62</v>
       </c>
-      <c r="R19">
+      <c r="T19">
         <v>2.72</v>
       </c>
-      <c r="S19">
+      <c r="U19">
         <v>0.08</v>
       </c>
-      <c r="T19">
+      <c r="V19">
         <v>97.4</v>
       </c>
-      <c r="U19" t="s">
-        <v>47</v>
-      </c>
-      <c r="V19" t="s">
-        <v>47</v>
-      </c>
       <c r="W19" t="s">
+        <v>47</v>
+      </c>
+      <c r="X19" t="s">
+        <v>47</v>
+      </c>
+      <c r="Y19" t="s">
         <v>49</v>
       </c>
-      <c r="X19" t="s">
+      <c r="Z19" t="s">
         <v>48</v>
       </c>
-      <c r="Y19" t="s">
-        <v>47</v>
-      </c>
-      <c r="Z19" t="s">
-        <v>47</v>
-      </c>
       <c r="AA19" t="s">
         <v>47</v>
       </c>
+      <c r="AB19" t="s">
+        <v>47</v>
+      </c>
+      <c r="AC19" t="s">
+        <v>47</v>
+      </c>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -2295,15 +2356,9 @@
       <c r="F20">
         <v>-85.971446999999998</v>
       </c>
-      <c r="G20" t="s">
+      <c r="I20" t="s">
         <v>51</v>
       </c>
-      <c r="H20" t="s">
-        <v>54</v>
-      </c>
-      <c r="I20" t="s">
-        <v>54</v>
-      </c>
       <c r="J20" t="s">
         <v>54</v>
       </c>
@@ -2359,10 +2414,16 @@
         <v>54</v>
       </c>
       <c r="AB20" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD20" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2378,15 +2439,9 @@
       <c r="F21">
         <v>-85.958196000000001</v>
       </c>
-      <c r="G21" t="s">
+      <c r="I21" t="s">
         <v>51</v>
       </c>
-      <c r="H21" t="s">
-        <v>54</v>
-      </c>
-      <c r="I21" t="s">
-        <v>54</v>
-      </c>
       <c r="J21" t="s">
         <v>54</v>
       </c>
@@ -2442,11 +2497,17 @@
         <v>54</v>
       </c>
       <c r="AB21" t="s">
+        <v>54</v>
+      </c>
+      <c r="AC21" t="s">
+        <v>54</v>
+      </c>
+      <c r="AD21" t="s">
         <v>55</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AA1" xr:uid="{22E256C1-2401-41CC-88F3-2A60CDB12830}"/>
+  <autoFilter ref="A1:AC1" xr:uid="{22E256C1-2401-41CC-88F3-2A60CDB12830}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>